<commit_message>
Aplicatie cu Front+back functional
Frontend+Backend cu functional care merge
trebuie ajustat o interfata placuta pentru utilizatori
folderul frontend se pune in examsch
va arata asa directorul:
examsch->frontend ,
examsch->exam_app
</commit_message>
<xml_diff>
--- a/vizualizare_date/sefgrupe.xlsx
+++ b/vizualizare_date/sefgrupe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VadimPK\Desktop\examsch\exam_app\vizualizare_date\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA88087A-2498-46A7-9DCF-071AC397118E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03685FFE-09EF-42CC-8161-4F656939602D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1320" windowWidth="13980" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3945" yWindow="2055" windowWidth="20025" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -518,7 +518,7 @@
         <v>33</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
         <v>29</v>

</xml_diff>